<commit_message>
Fix banner size (#230)
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/BannerTests.DictionarySheetBanner.verified.xlsx
+++ b/src/Excelsior.Tests/BannerTests.DictionarySheetBanner.verified.xlsx
@@ -54,7 +54,7 @@
     <col min="2" max="2" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Imported data - do not edit.</t>
@@ -88,7 +88,7 @@
   </sheetData>
   <autoFilter ref="A2:B3"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A1:XFD1"/>
   </mergeCells>
 </worksheet>
 </file>

</xml_diff>